<commit_message>
add all aviation files and changes
</commit_message>
<xml_diff>
--- a/SetRules.xlsx
+++ b/SetRules.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rbsul\Documents\GitHub\times-ireland-model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84D31DBA-173C-4BC5-ABF7-FAC6E95B136D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{100D1D2D-565A-4C16-BEBB-B2DC122AEAAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="16" r:id="rId1"/>
@@ -109,7 +109,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1956" uniqueCount="729">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1857" uniqueCount="684">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -2161,141 +2161,6 @@
   </si>
   <si>
     <t>S*,FT-SUP*,IMP*,EXP*,MIN*,-S-*,,-IMP*Z</t>
-  </si>
-  <si>
-    <t>RSD_BLD-ATT-HP</t>
-  </si>
-  <si>
-    <t>RSD_BLD-ATT-ELC</t>
-  </si>
-  <si>
-    <t>RSD_BLD-ATT-GAS</t>
-  </si>
-  <si>
-    <t>RSD_BLD-ATT-OTH</t>
-  </si>
-  <si>
-    <t>RSD_BLD-APT-HP</t>
-  </si>
-  <si>
-    <t>RSD_BLD-APT-ELC</t>
-  </si>
-  <si>
-    <t>RSD_BLD-APT-GAS</t>
-  </si>
-  <si>
-    <t>RSD_BLD-APT-OTH</t>
-  </si>
-  <si>
-    <t>RSD_BLD-DET-HP</t>
-  </si>
-  <si>
-    <t>RSD_BLD-DET-ELC</t>
-  </si>
-  <si>
-    <t>RSD_BLD-DET-GAS</t>
-  </si>
-  <si>
-    <t>RSD_BLD-DET-OTH</t>
-  </si>
-  <si>
-    <t>Residential - Attached - Heat pumps</t>
-  </si>
-  <si>
-    <t>Residential - Detached - Heat pumps</t>
-  </si>
-  <si>
-    <t>Residential - Attached - Electric</t>
-  </si>
-  <si>
-    <t>Residential - Attached - Gas</t>
-  </si>
-  <si>
-    <t>Residential - Attached - Other</t>
-  </si>
-  <si>
-    <t>Residential - Apartments - Heat pumps</t>
-  </si>
-  <si>
-    <t>Residential - Apartments - Electric</t>
-  </si>
-  <si>
-    <t>Residential - Apartments - Gas</t>
-  </si>
-  <si>
-    <t>Residential - Apartments - Other</t>
-  </si>
-  <si>
-    <t>Residential - Detached - Electric</t>
-  </si>
-  <si>
-    <t>Residential - Detached - Gas</t>
-  </si>
-  <si>
-    <t>Residential - Detached - Other</t>
-  </si>
-  <si>
-    <t>R*ATT*HPN*</t>
-  </si>
-  <si>
-    <t>R*DET*HPN*</t>
-  </si>
-  <si>
-    <t>R*SH*ATT*GAS*,R*SW*ATT*GAS*</t>
-  </si>
-  <si>
-    <t>R*SH*DET*GAS*,R*SW*DET*GAS*</t>
-  </si>
-  <si>
-    <t>R*SH*ATT*,R*SW*ATT*</t>
-  </si>
-  <si>
-    <t>R*APT*HPN*</t>
-  </si>
-  <si>
-    <t>R*SH*APT*GAS*,R*SW*APT*GAS*</t>
-  </si>
-  <si>
-    <t>R*SH*APT*,R*SW*APT*</t>
-  </si>
-  <si>
-    <t>R*SH*DET*,R*SW*DET*</t>
-  </si>
-  <si>
-    <t>R*SH*ATT*ELC*,-R*HPN*</t>
-  </si>
-  <si>
-    <t>R*SH*APT*ELC*,-R*HPN*</t>
-  </si>
-  <si>
-    <t>R*SH*DET*ELC*,-R*HPN*</t>
-  </si>
-  <si>
-    <t>P*STG*BA*</t>
-  </si>
-  <si>
-    <t>P*STG*PS*</t>
-  </si>
-  <si>
-    <t>STR-BAT</t>
-  </si>
-  <si>
-    <t>STR-PH</t>
-  </si>
-  <si>
-    <t>Electricity Storage -  Batteries</t>
-  </si>
-  <si>
-    <t>Electricity Storage -  Pumped hydro</t>
-  </si>
-  <si>
-    <t>*H2*STG*</t>
-  </si>
-  <si>
-    <t>STR-H2</t>
-  </si>
-  <si>
-    <t>Hydrogen Storage - underground</t>
   </si>
 </sst>
 </file>
@@ -6697,17 +6562,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A254A0F-7158-4F85-B7C3-36851FAE9E89}">
   <sheetPr codeName="Sheet10"/>
   <dimension ref="A1:Z99"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="4" width="21.7109375" customWidth="1"/>
-    <col min="5" max="6" width="14.140625" customWidth="1"/>
-    <col min="7" max="7" width="12.140625" customWidth="1"/>
-    <col min="8" max="10" width="8.140625" customWidth="1"/>
-    <col min="11" max="11" width="9.7109375" customWidth="1"/>
-    <col min="12" max="12" width="8.140625" customWidth="1"/>
+    <col min="1" max="4" width="21.7265625" customWidth="1"/>
+    <col min="5" max="6" width="14.1796875" customWidth="1"/>
+    <col min="7" max="7" width="12.1796875" customWidth="1"/>
+    <col min="8" max="10" width="8.1796875" customWidth="1"/>
+    <col min="11" max="11" width="9.7265625" customWidth="1"/>
+    <col min="12" max="12" width="8.1796875" customWidth="1"/>
     <col min="13" max="13" width="10" customWidth="1"/>
-    <col min="14" max="14" width="11.42578125" customWidth="1"/>
-    <col min="15" max="15" width="13.42578125" customWidth="1"/>
+    <col min="14" max="14" width="11.453125" customWidth="1"/>
+    <col min="15" max="15" width="13.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26">
@@ -9544,12 +9409,12 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:L19"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="57.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="57.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -10061,10 +9926,10 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:J83"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="4" max="4" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="40.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="40.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -12221,10 +12086,10 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:L20"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="6" max="6" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="40.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -12713,10 +12578,10 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:P36"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="6" max="6" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="40.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="40.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -13776,13 +13641,13 @@
   <sheetPr codeName="Sheet4">
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:L22"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="49" customWidth="1"/>
-    <col min="5" max="5" width="34.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="67.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="41.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="34.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="67.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -14325,294 +14190,6 @@
         <v>15</v>
       </c>
       <c r="K22" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11">
-      <c r="B23" t="s">
-        <v>708</v>
-      </c>
-      <c r="F23" t="s">
-        <v>684</v>
-      </c>
-      <c r="G23" t="s">
-        <v>696</v>
-      </c>
-      <c r="H23" t="s">
-        <v>15</v>
-      </c>
-      <c r="I23" t="s">
-        <v>16</v>
-      </c>
-      <c r="J23" t="s">
-        <v>15</v>
-      </c>
-      <c r="K23" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11">
-      <c r="B24" t="s">
-        <v>717</v>
-      </c>
-      <c r="F24" t="s">
-        <v>685</v>
-      </c>
-      <c r="G24" t="s">
-        <v>698</v>
-      </c>
-      <c r="H24" t="s">
-        <v>15</v>
-      </c>
-      <c r="I24" t="s">
-        <v>16</v>
-      </c>
-      <c r="J24" t="s">
-        <v>15</v>
-      </c>
-      <c r="K24" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11">
-      <c r="B25" t="s">
-        <v>710</v>
-      </c>
-      <c r="F25" t="s">
-        <v>686</v>
-      </c>
-      <c r="G25" t="s">
-        <v>699</v>
-      </c>
-      <c r="H25" t="s">
-        <v>15</v>
-      </c>
-      <c r="I25" t="s">
-        <v>16</v>
-      </c>
-      <c r="J25" t="s">
-        <v>15</v>
-      </c>
-      <c r="K25" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11">
-      <c r="A26" t="str">
-        <f>"-"&amp;F23&amp;",-"&amp;F24&amp;",-"&amp;F25</f>
-        <v>-RSD_BLD-ATT-HP,-RSD_BLD-ATT-ELC,-RSD_BLD-ATT-GAS</v>
-      </c>
-      <c r="B26" t="s">
-        <v>712</v>
-      </c>
-      <c r="F26" t="s">
-        <v>687</v>
-      </c>
-      <c r="G26" t="s">
-        <v>700</v>
-      </c>
-      <c r="H26" t="s">
-        <v>15</v>
-      </c>
-      <c r="I26" t="s">
-        <v>16</v>
-      </c>
-      <c r="J26" t="s">
-        <v>15</v>
-      </c>
-      <c r="K26" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11">
-      <c r="B27" t="s">
-        <v>713</v>
-      </c>
-      <c r="F27" t="s">
-        <v>688</v>
-      </c>
-      <c r="G27" t="s">
-        <v>701</v>
-      </c>
-      <c r="H27" t="s">
-        <v>15</v>
-      </c>
-      <c r="I27" t="s">
-        <v>16</v>
-      </c>
-      <c r="J27" t="s">
-        <v>15</v>
-      </c>
-      <c r="K27" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11">
-      <c r="B28" t="s">
-        <v>718</v>
-      </c>
-      <c r="F28" t="s">
-        <v>689</v>
-      </c>
-      <c r="G28" t="s">
-        <v>702</v>
-      </c>
-      <c r="H28" t="s">
-        <v>15</v>
-      </c>
-      <c r="I28" t="s">
-        <v>16</v>
-      </c>
-      <c r="J28" t="s">
-        <v>15</v>
-      </c>
-      <c r="K28" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11">
-      <c r="B29" t="s">
-        <v>714</v>
-      </c>
-      <c r="F29" t="s">
-        <v>690</v>
-      </c>
-      <c r="G29" t="s">
-        <v>703</v>
-      </c>
-      <c r="H29" t="s">
-        <v>15</v>
-      </c>
-      <c r="I29" t="s">
-        <v>16</v>
-      </c>
-      <c r="J29" t="s">
-        <v>15</v>
-      </c>
-      <c r="K29" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11">
-      <c r="A30" t="str">
-        <f>"-"&amp;F27&amp;",-"&amp;F28&amp;",-"&amp;F29</f>
-        <v>-RSD_BLD-APT-HP,-RSD_BLD-APT-ELC,-RSD_BLD-APT-GAS</v>
-      </c>
-      <c r="B30" t="s">
-        <v>715</v>
-      </c>
-      <c r="F30" t="s">
-        <v>691</v>
-      </c>
-      <c r="G30" t="s">
-        <v>704</v>
-      </c>
-      <c r="H30" t="s">
-        <v>15</v>
-      </c>
-      <c r="I30" t="s">
-        <v>16</v>
-      </c>
-      <c r="J30" t="s">
-        <v>15</v>
-      </c>
-      <c r="K30" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11">
-      <c r="B31" t="s">
-        <v>709</v>
-      </c>
-      <c r="F31" t="s">
-        <v>692</v>
-      </c>
-      <c r="G31" t="s">
-        <v>697</v>
-      </c>
-      <c r="H31" t="s">
-        <v>15</v>
-      </c>
-      <c r="I31" t="s">
-        <v>16</v>
-      </c>
-      <c r="J31" t="s">
-        <v>15</v>
-      </c>
-      <c r="K31" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11">
-      <c r="B32" t="s">
-        <v>719</v>
-      </c>
-      <c r="F32" t="s">
-        <v>693</v>
-      </c>
-      <c r="G32" t="s">
-        <v>705</v>
-      </c>
-      <c r="H32" t="s">
-        <v>15</v>
-      </c>
-      <c r="I32" t="s">
-        <v>16</v>
-      </c>
-      <c r="J32" t="s">
-        <v>15</v>
-      </c>
-      <c r="K32" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11">
-      <c r="B33" t="s">
-        <v>711</v>
-      </c>
-      <c r="F33" t="s">
-        <v>694</v>
-      </c>
-      <c r="G33" t="s">
-        <v>706</v>
-      </c>
-      <c r="H33" t="s">
-        <v>15</v>
-      </c>
-      <c r="I33" t="s">
-        <v>16</v>
-      </c>
-      <c r="J33" t="s">
-        <v>15</v>
-      </c>
-      <c r="K33" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11">
-      <c r="A34" t="str">
-        <f>"-"&amp;F31&amp;",-"&amp;F32&amp;",-"&amp;F33</f>
-        <v>-RSD_BLD-DET-HP,-RSD_BLD-DET-ELC,-RSD_BLD-DET-GAS</v>
-      </c>
-      <c r="B34" t="s">
-        <v>716</v>
-      </c>
-      <c r="F34" t="s">
-        <v>695</v>
-      </c>
-      <c r="G34" t="s">
-        <v>707</v>
-      </c>
-      <c r="H34" t="s">
-        <v>15</v>
-      </c>
-      <c r="I34" t="s">
-        <v>16</v>
-      </c>
-      <c r="J34" t="s">
-        <v>15</v>
-      </c>
-      <c r="K34" t="s">
         <v>16</v>
       </c>
     </row>
@@ -14627,10 +14204,10 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:L38"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="6" max="6" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="58.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="58.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -15730,11 +15307,11 @@
   <sheetPr codeName="Sheet6">
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:L19"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="6" max="6" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="53.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="53.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -16078,57 +15655,6 @@
         <v>15</v>
       </c>
       <c r="I19" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="20" spans="2:9">
-      <c r="B20" t="s">
-        <v>720</v>
-      </c>
-      <c r="F20" t="s">
-        <v>722</v>
-      </c>
-      <c r="G20" t="s">
-        <v>724</v>
-      </c>
-      <c r="H20" t="s">
-        <v>15</v>
-      </c>
-      <c r="I20" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="21" spans="2:9">
-      <c r="B21" t="s">
-        <v>721</v>
-      </c>
-      <c r="F21" t="s">
-        <v>723</v>
-      </c>
-      <c r="G21" t="s">
-        <v>725</v>
-      </c>
-      <c r="H21" t="s">
-        <v>15</v>
-      </c>
-      <c r="I21" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="22" spans="2:9">
-      <c r="B22" t="s">
-        <v>726</v>
-      </c>
-      <c r="F22" t="s">
-        <v>727</v>
-      </c>
-      <c r="G22" t="s">
-        <v>728</v>
-      </c>
-      <c r="H22" t="s">
-        <v>15</v>
-      </c>
-      <c r="I22" t="s">
         <v>16</v>
       </c>
     </row>
@@ -16143,10 +15669,10 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:L3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="6" max="6" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="53.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="53.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -16230,10 +15756,10 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:L3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="6" max="6" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="53.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="53.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">

</xml_diff>